<commit_message>
L2 + L3 lifecycle contracts ratified and landed as registry Lifecycle sheets (L4 inherits: human-mint CREATE only)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BAgZi4RCB3bWFG5MSWcW8V
</commit_message>
<xml_diff>
--- a/AIVIA_Design/L1_KG2_Logic_Layer_Registry_DRAFT.xlsx
+++ b/AIVIA_Design/L1_KG2_Logic_Layer_Registry_DRAFT.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Edge_Types" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Rules_to_Checks" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Fixture_Families" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Lifecycle" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1056,4 +1057,156 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Writer / trigger</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Postconditions</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>CREATE</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>the MAPPER only; estate file intake (trigger cites the estate-source seam — H3 uncontracted)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>full tree per metamodel; conservation handled ⊎ remainder = total; evidence on every node; resolution complete (edges or counted); name-keyed identities minted</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>LC2-C1 authored file -&gt; authored tree · LC2-C2 unmappable construct -&gt; counted remainder, tree whole · LC2-C3 unresolvable ref -&gt; no edge, counted</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SUPERSEDE</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>the mapper; re-parse of a known source path</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>new tree version appended, prior retired; name-keyed identities stable where names persist; content-key drift as evidence; attachments to persisting names undisturbed. resolves_to binds to IDENTITY not version — L1 supersession needs zero re-resolution</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>LC2-S1 edit inside scope -&gt; identity + attachment survive, drift flagged (= scenario S1) · LC2-S2 rename -&gt; old retired, new minted, attachment surfaces for human re-attach · LC2-S3 unchanged file -&gt; no new version</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>RETIRE</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>the mapper; source path absent from estate</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>whole tree retired, never removed; attachments surface</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>LC2-R1 deleted file -&gt; retired tree + surfaced attachments</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>READ</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>anyone</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>current-vs-retired explicit; completeness declared</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>LC2-D1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>FORBIDDEN</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>any writer but mapper (LC2-F1 census) · text-derived structure (LC2-F2 parser-authority plank) · hand edits (LC2-F3) · physical delete (LC2-F4) · partial parse shipped whole (LC2-F5 — conservation IS the atomicity)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>